<commit_message>
Record the three calendar dates on the phone.
19 Mar, 14 Sep and 11 Oct match the exported year, and the month still opens with no network. No override was added.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M4-calendar.xlsx
+++ b/tests/M4-calendar.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -454,6 +454,7 @@
     <col width="24.140625" customWidth="1" min="7" max="7"/>
     <col width="26.5703125" customWidth="1" min="8" max="8"/>
     <col width="30.42578125" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +513,11 @@
           <t>Test Type</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Result</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="57.95" customHeight="1">
       <c r="A2" s="3" t="n">
@@ -557,6 +563,11 @@
       </c>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS on the phone. 19 Mar 2026 shows Thu 19 Mar, kṛṣṇa amāvāsyā, Hyderabad, and no observance card. The Hyderabad CSV has tithi 15, kṛṣṇa, Phālguna, and no observance.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="57.95" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -602,6 +613,11 @@
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. 14 Sep 2026 shows Vinayaka Chavithi. The CSV has śukla 3, Bhādrapada, obs.vinayaka-chavithi.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.95" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -646,6 +662,11 @@
       </c>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. 11 Oct 2026 shows Sun 11 Oct, śukla pratipat, Hyderabad, and no observance card. The CSV has śukla 1, Āśvayuja, and no observance.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.95" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -689,6 +710,11 @@
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hyderabad and Vijayawada 2026 CSVs are in tests/calendar-export. The three dates match the phone. Comparison with the TTD panchangam is still open, so no override was added.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="57.95" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -777,6 +803,11 @@
       </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Day 14 opens the Vinayaka Chavithi page. What families do is open, and the katha card is under it.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="57.95" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -1176,6 +1207,11 @@
       </c>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. With airplane mode on and no network, the calendar month still opens.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>